<commit_message>
Anyag- és élzáró-termékjavaslat (21 jelölt, forrással, áras) az Excelben, asztalosi üzenet tervezete, csomag frissítve
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Y3AFi4uRByLtwt7ksfcxj
</commit_message>
<xml_diff>
--- a/execution/a902-s01-kyoto-ink-20261026/R16_GYARTAS/40_F3F4_dokumentacio/R16_J_szabasjegyzek.xlsx
+++ b/execution/a902-s01-kyoto-ink-20261026/R16_GYARTAS/40_F3F4_dokumentacio/R16_J_szabasjegyzek.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Vasalat" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Furatok" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Nyitott és jelmagyarázat" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Anyagjavaslat" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6777" uniqueCount="1248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6908" uniqueCount="1339">
   <si>
     <t xml:space="preserve">Címke-ID (MPR alap)</t>
   </si>
@@ -3802,6 +3803,287 @@
   </si>
   <si>
     <t xml:space="preserve">Lapanyag/dekor termék és táblaméret; élzáró vastagság és előmarás; polctartó típus; fiók sín furatképe; LED-profilok; helyszíni felmérés.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anyagkód</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gyártó</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Termékkód</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Név</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Felület</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Táblaméret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Élzáró (ABS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forgalmazó</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ár</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ár egység / megjegyzés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ár dátuma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Színegyezés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Egger (hordozó) + IVM Chemicals / Milesi (2K PU)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Egger MDF natúr 18 mm + Milesi LBR 30 2K PU MDF-alapozó (LNB 42 edző) + Milesi PU pigmentált matt fedő NCS S 7005-Y20R-re keverve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matt bronzbarna festett MDF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2K PU matt (fényfok egyeztetendő)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2800x2070</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MDF: Lapp-fa Kft.; festék: M.L.S. Magyarország Kft. (Szigetszentmiklós)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ft/tábla (MDF) nettó; festék ár nincs nyilvános</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Az NCS S 7005-Y20R kódot az Egger U741 Láva szürke referenciájaként is megadja (RAL 7013 közelítés) – így a festett R16 M01 és a laminált U741 ugyanabba a színcsaládba esik; a 'bronzbarna' hatás a kevert festékmintán ellenőrizendő. Fedőfesték-cikkszám a forgalmazótól.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://lapp-fa.hu/mdf/mdf-egger-natur-18mm-2800x2070-141.html
+https://www.milesi.hu/ipari-felhasznalok/component/pes/product/66?catid=2212</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JAVASLAT – mintával ellenőrizendő</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sayerlack (Sherwin-Williams)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2K PU pigmentált rendszer, NCS S 7005-Y20R – cikkszám a forgalmazótól</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alternatív festékrendszer Egger MDF 18 mm-re</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2K PU matt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mile Color Kft. (Miskolc) / Lakgruppen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ár nincs nyilvános; termékkód nem igazolt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://sayerlack.hu/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vescom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bely+Print 1040.01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bely+Print – digitálisan nyomtatott vinyl falburkolat len (linen) textúrával</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vinyl, len textúra; kb. 350 g/m², szélesség 134 cm (nyomtatható 133 cm); MDF-re kasírozva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tekercs 1340 mm széles + 18 mm MDF hordozó (Egger MDF 2800x2070)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Top Trade Kft. (Vescom-márkát forgalmaz; 1142 Bp., Erzsébet királyné útja 125.) – a Bely+Print HU-elérhetősége nem igazolt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHF (egység nincs jelölve; 'Price on request' is szerepel) nincs jelölve (wirzwelt.ch, CH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LÉTEZIK: az 1040.01 a Bely+Print (nyomtatható) alapcikk kódja; a végső szín a digitális nyomattól függ, minimum rendelés 'custom'. Nem raktári lapanyag: tekercs, amit MDF-re kell kasírozni (asztalos/kasírozó), élzárása külön megoldandó. HU ár nincs nyilvános – Top Trade-től kérendő.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://vescom.com/en/products/belyprint
+https://wirzwelt.ch/en/vescom-wallcovering-print-bely-print-pro-1040-01pro
+https://kubecontract.com/products/pleso-print
+https://toptrade.hu/vescom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Egger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F433 ST10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anthracite Linen / Antracit len</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST10 Deepskin Rough – finom len hatás</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Egger · ABS F433 ST10 (cikkszám a forgalmazótól)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forest Hungary (cikksz. 20030433180) / Lapszabo.hu (Woodframe Kft.) / Szabhatjuk.hu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ft/tábla (szabott táblaár) bruttó (lapszabo.hu)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kész lapanyag-alternatíva textilhatással, kasírozás nélkül. Világosabb textil-alternatíva: Egger F416 ST10 Bézs textil (lásd S16 M04/2). Színegyezés a Vescom nyomathoz nem értelmezhető – mintával.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.foresteu.com/laptermekek-es-tartozekaik/butorlap/egger-fantazia/20030433180-butorlap-egger-fantazia-f433-st10-antracit-len-2800x2070x18mm
+https://www.lapszabo.hu/butorlap/egger/f433-st10-antracit-len
+https://www.egger.com/en/interior/decor-detail/F433_10?country=GB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U741 ST9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lava Grey / Láva szürke – korpusz belső</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST9 Smoothtouch Matt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Egger · ABS E_U741 ST9 – 0,8/23 mm (24744/0741)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lapp-fa Kft. (XVII. ker. készleten) / Fabuli / JAF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ft/tábla nettó (Lapp-fa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Becslés: NCS S 7005-Y20R – azonos az R16 M01 festék célszínével, ezért a belső és a festett külső egy tónusban marad; egyben egységesíti az S16 M01-gyel a beszerzést. 8 mm-es U741 változatot HU-ban nem találtam (JAF csak 18 mm-t listáz) – 8 mm-re lásd 2. jelölt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://lapp-fa.hu/butorlap/u-741-st9-lava-szurke-18mm-2800x2070-154.html
+https://fabuli.hu/butorlap-egger-uni-u741-st9-lava-szurke-2800x2070x18mm-7646
+https://www.egger.com/en/interior/decor-detail/U741_9?country=GB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U961 ST2 (8 mm) / U963 ST9 (16 mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 mm-es korpusz/hátlap változat – ugyanaz, mint S16 M08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST2 / ST9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8, 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lásd S16 M08 – HU 8 mm rendelhetőség ellenőrizendő</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ár nincs nyilvános. Grafit, nem láva tónus – ha a 8 mm-es elem látszik, színeltérés; ha nem látszik, elfogadható. Alternatíva: 8 mm MDF festve (R16 M01 rendszerrel).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lawcris.co.uk/2800mm-x-2070mm-x-8mm-u961-st2-graphite-grey-melamine-faced-chipboard-cmeu961st208</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ismeretlen (Alföldfa saját forgalom)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bükk (enyhén gőzölt) táblásított lap 18 mm, AB, HT (hossztoldott)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 mm bükk táblásított lap – asztalos hasítja 18×18 mm-es lécre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nyers, csiszolt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3000x1200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alföldfa (5000 Szolnok); rendelésre, 8–10 munkanap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ft/tábla bruttó (árlista érvényes 2026-10-30-ig – lejár, újrakérendő)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kész 18×18 mm-es gyalult bükk lécet HU webshopban nem találtam (OBI-nál 18 mm-es kerek bükk rúd van, az nem jó). HT = hossztoldott – látszó lécnél a 2000x1200 'TM' (64 900 Ft bruttó) változat toldásmentességét kérdezd meg. Jobb: asztalos saját bükk pallóból hasítja.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.alfoldfa.hu/termek/bukk-tablasitott-lap/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ismeretlen (finn nyír, márka nincs kitöltve)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rétegelt finn nyír 18 mm BB/CP, vízálló ragasztású</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 mm nyír rétegelt lemez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BB/CP (BBWG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2500x1250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lapp-fa Kft. (Budapest XVII. ker. / központi raktár)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ft/tábla nettó (egység a forrásban nincs kiírva, táblaár valószínű)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP hátoldal javításokkal – ha mindkét oldal látszik, BB/BB minőség kell (pl. OKFT 1525x1525x18 BB/BB).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://lapp-fa.hu/retegeltlemez/retegelt-finn-nyir-18-mm-2500x1250-bb-cp-vizallo-ragasztasu-1838.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ismeretlen (nyír, BFU-100)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nyír rétegelt lemez 15 mm BB/WG, BFU-100, 11 réteg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 mm nyír rétegelt fiókdobozhoz (azonos az S16 M07-tel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">csiszolt mindkét oldal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OKFT Faáruház (Algyő)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ft/tábla nincs jelölve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ugyanaz a tétel, mint S16 M07 – közös beszerzés javasolt. Budapesti 15 mm-es forrást nem találtam (Lapp-fa csak 18 mm-t listáz).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.okftfaaruhaz.hu/NYIR-RET-LEM-15mm-BB/WG-vizallo-2500x1250x15mm-BFU</t>
   </si>
 </sst>
 </file>
@@ -3936,7 +4218,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3983,6 +4265,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -48889,4 +49175,515 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:P10"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>518</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1249</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1250</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1251</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1252</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>1253</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>1254</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>1255</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>1256</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>1257</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>1258</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>1260</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>1261</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>1262</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>1263</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12" t="s">
+        <v>1266</v>
+      </c>
+      <c r="K2" s="12" t="n">
+        <v>21694</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>1267</v>
+      </c>
+      <c r="M2" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="N2" s="12" t="s">
+        <v>1269</v>
+      </c>
+      <c r="O2" s="12" t="s">
+        <v>1270</v>
+      </c>
+      <c r="P2" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>1272</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>1273</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>1274</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>1275</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12" t="s">
+        <v>1276</v>
+      </c>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12" t="s">
+        <v>1277</v>
+      </c>
+      <c r="O3" s="12" t="s">
+        <v>1278</v>
+      </c>
+      <c r="P3" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>1279</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>1280</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>1281</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>1282</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>1283</v>
+      </c>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>99.56</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>1285</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="N4" s="12" t="s">
+        <v>1286</v>
+      </c>
+      <c r="O4" s="12" t="s">
+        <v>1287</v>
+      </c>
+      <c r="P4" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>1289</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>1290</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>1291</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>1292</v>
+      </c>
+      <c r="J5" s="12" t="s">
+        <v>1293</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>67089</v>
+      </c>
+      <c r="L5" s="12" t="s">
+        <v>1294</v>
+      </c>
+      <c r="M5" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="N5" s="12" t="s">
+        <v>1295</v>
+      </c>
+      <c r="O5" s="12" t="s">
+        <v>1296</v>
+      </c>
+      <c r="P5" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>1297</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>1298</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>1299</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>1300</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>1301</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>29629</v>
+      </c>
+      <c r="L6" s="12" t="s">
+        <v>1302</v>
+      </c>
+      <c r="M6" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="N6" s="12" t="s">
+        <v>1303</v>
+      </c>
+      <c r="O6" s="12" t="s">
+        <v>1304</v>
+      </c>
+      <c r="P6" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>1305</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>1306</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>1307</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>1308</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>1265</v>
+      </c>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12" t="s">
+        <v>1309</v>
+      </c>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12" t="s">
+        <v>1310</v>
+      </c>
+      <c r="O7" s="12" t="s">
+        <v>1311</v>
+      </c>
+      <c r="P7" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>1312</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>1313</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>1314</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>1315</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>1316</v>
+      </c>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12" t="s">
+        <v>1317</v>
+      </c>
+      <c r="K8" s="12" t="n">
+        <v>71900</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>1318</v>
+      </c>
+      <c r="M8" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>1319</v>
+      </c>
+      <c r="O8" s="12" t="s">
+        <v>1320</v>
+      </c>
+      <c r="P8" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>1321</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>1322</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>1323</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>1324</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>1325</v>
+      </c>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12" t="s">
+        <v>1326</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>34960</v>
+      </c>
+      <c r="L9" s="12" t="s">
+        <v>1327</v>
+      </c>
+      <c r="M9" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="N9" s="12" t="s">
+        <v>1328</v>
+      </c>
+      <c r="O9" s="12" t="s">
+        <v>1329</v>
+      </c>
+      <c r="P9" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>1330</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>1331</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>1332</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>1333</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>1334</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>1325</v>
+      </c>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12" t="s">
+        <v>1335</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>38821</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>1336</v>
+      </c>
+      <c r="M10" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="N10" s="12" t="s">
+        <v>1337</v>
+      </c>
+      <c r="O10" s="12" t="s">
+        <v>1338</v>
+      </c>
+      <c r="P10" s="12" t="s">
+        <v>1271</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
R15C + v8: D6 fiók 35 mm-rel feljebb, anyag- és ABS-döntések (U741/0,8, H1399/2 mm, F424 HPL, R16 F433, egy darabos fedő) – 129/129, 106/106
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Y3AFi4uRByLtwt7ksfcxj
</commit_message>
<xml_diff>
--- a/execution/a902-s01-kyoto-ink-20261026/R16_GYARTAS/40_F3F4_dokumentacio/R16_J_szabasjegyzek.xlsx
+++ b/execution/a902-s01-kyoto-ink-20261026/R16_GYARTAS/40_F3F4_dokumentacio/R16_J_szabasjegyzek.xlsx
@@ -184,7 +184,7 @@
     <t xml:space="preserve">V</t>
   </si>
   <si>
-    <t xml:space="preserve">ABS 1 mm dekoregyező (korpusz)</t>
+    <t xml:space="preserve">ABS 0,8 mm Egger U741 ST9 (korpusz)</t>
   </si>
   <si>
     <t xml:space="preserve">E1+E4</t>
@@ -4737,13 +4737,13 @@
         <v>2330</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>2330</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M2" s="2" t="n">
         <v>2330</v>
@@ -4834,13 +4834,13 @@
         <v>2330</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>2330</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M3" s="2" t="n">
         <v>2330</v>
@@ -4934,13 +4934,13 @@
         <v>684</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="L4" s="2" t="n">
         <v>684</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>1</v>
@@ -5029,13 +5029,13 @@
         <v>684</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>684</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>1</v>
@@ -5123,13 +5123,13 @@
         <v>2294</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>353</v>
+        <v>353.2</v>
       </c>
       <c r="K6" s="2" t="n">
         <v>2294</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>354</v>
+        <v>354.2</v>
       </c>
       <c r="M6" s="2" t="n">
         <v>2294</v>
@@ -5221,13 +5221,13 @@
         <v>331</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>1</v>
@@ -5316,13 +5316,13 @@
         <v>331</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>1</v>
@@ -5411,13 +5411,13 @@
         <v>331</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>1</v>
@@ -5506,13 +5506,13 @@
         <v>331</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M10" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>1</v>
@@ -5601,13 +5601,13 @@
         <v>331</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>1</v>
@@ -5696,13 +5696,13 @@
         <v>331</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>1</v>
@@ -5791,13 +5791,13 @@
         <v>331</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L13" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>1</v>
@@ -5886,13 +5886,13 @@
         <v>331</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L14" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>1</v>
@@ -5981,13 +5981,13 @@
         <v>331</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>1</v>
@@ -6076,13 +6076,13 @@
         <v>331</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>289</v>
+        <v>289.2</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>331</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>290</v>
+        <v>290.2</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>1</v>
@@ -7421,13 +7421,13 @@
         <v>382</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L30" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M30" s="2" t="n">
         <v>382</v>
@@ -7516,13 +7516,13 @@
         <v>382</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L31" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M31" s="2" t="n">
         <v>382</v>
@@ -7614,13 +7614,13 @@
         <v>684</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>684</v>
       </c>
       <c r="M32" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="N32" s="2" t="n">
         <v>1</v>
@@ -8660,13 +8660,13 @@
         <v>382</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K43" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M43" s="2" t="n">
         <v>382</v>
@@ -8755,13 +8755,13 @@
         <v>382</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M44" s="2" t="n">
         <v>382</v>
@@ -8853,13 +8853,13 @@
         <v>414</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>414</v>
       </c>
       <c r="M45" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="N45" s="2" t="n">
         <v>1</v>
@@ -9899,13 +9899,13 @@
         <v>382</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K56" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M56" s="2" t="n">
         <v>382</v>
@@ -9994,13 +9994,13 @@
         <v>382</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>382</v>
@@ -10092,13 +10092,13 @@
         <v>414</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>414</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="N58" s="2" t="n">
         <v>1</v>
@@ -11138,13 +11138,13 @@
         <v>382</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L69" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M69" s="2" t="n">
         <v>382</v>
@@ -11233,13 +11233,13 @@
         <v>382</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L70" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M70" s="2" t="n">
         <v>382</v>
@@ -11331,13 +11331,13 @@
         <v>1044</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>1044</v>
       </c>
       <c r="M71" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="N71" s="2" t="n">
         <v>1</v>
@@ -12377,13 +12377,13 @@
         <v>382</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L82" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M82" s="2" t="n">
         <v>382</v>
@@ -12472,13 +12472,13 @@
         <v>382</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L83" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M83" s="2" t="n">
         <v>382</v>
@@ -12570,13 +12570,13 @@
         <v>414</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="L84" s="2" t="n">
         <v>414</v>
       </c>
       <c r="M84" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="N84" s="2" t="n">
         <v>1</v>
@@ -13616,13 +13616,13 @@
         <v>382</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L95" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M95" s="2" t="n">
         <v>382</v>
@@ -13711,13 +13711,13 @@
         <v>382</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>382</v>
       </c>
       <c r="L96" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="M96" s="2" t="n">
         <v>382</v>
@@ -13809,13 +13809,13 @@
         <v>414</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>381</v>
+        <v>381.2</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>414</v>
       </c>
       <c r="M97" s="2" t="n">
-        <v>382</v>
+        <v>382.2</v>
       </c>
       <c r="N97" s="2" t="n">
         <v>1</v>

</xml_diff>